<commit_message>
Add CO outcomes, bloom taxonomy, per-student evaluate, analytics dashboard, 20 Java questions EN+TA, evaluation metrics
</commit_message>
<xml_diff>
--- a/Hypothesis/EvalAI_Score_Collection.xlsx
+++ b/Hypothesis/EvalAI_Score_Collection.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\25Mar\Hypothesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB5EF492-C4FB-4519-9EFD-E1EE9E9670D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC41CBC2-5FB2-49D6-91D3-B25A26EF01A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Score Entry" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,6 @@
     <sheet name="Instructions" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -115,19 +114,10 @@
     <t>Q8</t>
   </si>
   <si>
-    <t>Q8 — Add your question here</t>
-  </si>
-  <si>
     <t>Q9</t>
   </si>
   <si>
-    <t>Q9 — Add your question here</t>
-  </si>
-  <si>
     <t>Q10</t>
-  </si>
-  <si>
-    <t>Q10 — Add your question here</t>
   </si>
   <si>
     <t>EvalAI — Statistical Summary (Auto-Calculated)</t>
@@ -278,6 +268,15 @@
   </si>
   <si>
     <t>What is JVM?</t>
+  </si>
+  <si>
+    <t>What is a variable in Java?</t>
+  </si>
+  <si>
+    <t>What is the difference between int and double in Java?</t>
+  </si>
+  <si>
+    <t>What is the use of if-else in Java?</t>
   </si>
 </sst>
 </file>
@@ -614,32 +613,32 @@
     <xf numFmtId="0" fontId="21" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -955,7 +954,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="31" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="28"/>
@@ -968,7 +967,7 @@
       <c r="I1" s="28"/>
     </row>
     <row r="2" spans="1:9" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="31" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="28"/>
@@ -1014,7 +1013,7 @@
       <c r="A5" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="B5" s="27" t="s">
+      <c r="B5" s="30" t="s">
         <v>12</v>
       </c>
       <c r="C5" s="2" t="s">
@@ -1164,7 +1163,7 @@
       <c r="A11" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="27" t="s">
+      <c r="B11" s="30" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="2" t="s">
@@ -1314,8 +1313,8 @@
       <c r="A17" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="27" t="s">
-        <v>75</v>
+      <c r="B17" s="30" t="s">
+        <v>72</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>13</v>
@@ -1464,8 +1463,8 @@
       <c r="A23" s="29" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="27" t="s">
-        <v>76</v>
+      <c r="B23" s="30" t="s">
+        <v>73</v>
       </c>
       <c r="C23" s="2" t="s">
         <v>13</v>
@@ -1614,8 +1613,8 @@
       <c r="A29" s="29" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="27" t="s">
-        <v>77</v>
+      <c r="B29" s="30" t="s">
+        <v>74</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>13</v>
@@ -1764,8 +1763,8 @@
       <c r="A35" s="29" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="27" t="s">
-        <v>78</v>
+      <c r="B35" s="30" t="s">
+        <v>75</v>
       </c>
       <c r="C35" s="2" t="s">
         <v>13</v>
@@ -1914,8 +1913,8 @@
       <c r="A41" s="29" t="s">
         <v>24</v>
       </c>
-      <c r="B41" s="27" t="s">
-        <v>79</v>
+      <c r="B41" s="30" t="s">
+        <v>76</v>
       </c>
       <c r="C41" s="2" t="s">
         <v>13</v>
@@ -2064,8 +2063,8 @@
       <c r="A47" s="29" t="s">
         <v>25</v>
       </c>
-      <c r="B47" s="27" t="s">
-        <v>26</v>
+      <c r="B47" s="30" t="s">
+        <v>77</v>
       </c>
       <c r="C47" s="2" t="s">
         <v>13</v>
@@ -2073,17 +2072,23 @@
       <c r="D47" s="3">
         <v>9.5</v>
       </c>
-      <c r="E47" s="4"/>
-      <c r="F47" s="5" t="str">
+      <c r="E47" s="4">
+        <v>9.77</v>
+      </c>
+      <c r="F47" s="5">
         <f>IF(E47="","",E47-D47)</f>
-        <v/>
+        <v>0.26999999999999957</v>
       </c>
       <c r="G47" s="6" t="str">
         <f>IF(E47="","",IF(AND(E47&gt;=9,E47&lt;=10),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H47" s="7"/>
-      <c r="I47" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H47" s="7">
+        <v>0.98</v>
+      </c>
+      <c r="I47" s="8">
+        <v>0.94</v>
+      </c>
     </row>
     <row r="48" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="28"/>
@@ -2094,17 +2099,23 @@
       <c r="D48" s="3">
         <v>7.5</v>
       </c>
-      <c r="E48" s="4"/>
-      <c r="F48" s="5" t="str">
+      <c r="E48" s="4">
+        <v>7.14</v>
+      </c>
+      <c r="F48" s="5">
         <f>IF(E48="","",E48-D48)</f>
-        <v/>
+        <v>-0.36000000000000032</v>
       </c>
       <c r="G48" s="6" t="str">
         <f>IF(E48="","",IF(AND(E48&gt;=7,E48&lt;=9),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H48" s="7"/>
-      <c r="I48" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H48" s="7">
+        <v>0.81</v>
+      </c>
+      <c r="I48" s="8">
+        <v>0.96</v>
+      </c>
     </row>
     <row r="49" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="28"/>
@@ -2115,17 +2126,23 @@
       <c r="D49" s="3">
         <v>5.5</v>
       </c>
-      <c r="E49" s="4"/>
-      <c r="F49" s="5" t="str">
+      <c r="E49" s="4">
+        <v>7.18</v>
+      </c>
+      <c r="F49" s="5">
         <f>IF(E49="","",E49-D49)</f>
-        <v/>
+        <v>1.6799999999999997</v>
       </c>
       <c r="G49" s="6" t="str">
         <f>IF(E49="","",IF(AND(E49&gt;=4.5,E49&lt;=7),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H49" s="7"/>
-      <c r="I49" s="8"/>
+        <v>✗ No</v>
+      </c>
+      <c r="H49" s="7">
+        <v>0.89</v>
+      </c>
+      <c r="I49" s="8">
+        <v>0.99</v>
+      </c>
     </row>
     <row r="50" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="28"/>
@@ -2136,17 +2153,23 @@
       <c r="D50" s="3">
         <v>3.5</v>
       </c>
-      <c r="E50" s="4"/>
-      <c r="F50" s="5" t="str">
+      <c r="E50" s="4">
+        <v>6.75</v>
+      </c>
+      <c r="F50" s="5">
         <f>IF(E50="","",E50-D50)</f>
-        <v/>
+        <v>3.25</v>
       </c>
       <c r="G50" s="6" t="str">
         <f>IF(E50="","",IF(AND(E50&gt;=2.5,E50&lt;=4.5),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H50" s="7"/>
-      <c r="I50" s="8"/>
+        <v>✗ No</v>
+      </c>
+      <c r="H50" s="7">
+        <v>0.88</v>
+      </c>
+      <c r="I50" s="8">
+        <v>0.98</v>
+      </c>
     </row>
     <row r="51" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="28"/>
@@ -2157,17 +2180,23 @@
       <c r="D51" s="3">
         <v>1.5</v>
       </c>
-      <c r="E51" s="4"/>
-      <c r="F51" s="5" t="str">
+      <c r="E51" s="4">
+        <v>0.02</v>
+      </c>
+      <c r="F51" s="5">
         <f>IF(E51="","",E51-D51)</f>
-        <v/>
+        <v>-1.48</v>
       </c>
       <c r="G51" s="6" t="str">
         <f>IF(E51="","",IF(AND(E51&gt;=0,E51&lt;=2.5),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H51" s="7"/>
-      <c r="I51" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H51" s="7">
+        <v>0.81</v>
+      </c>
+      <c r="I51" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="52" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="13"/>
@@ -2182,10 +2211,10 @@
     </row>
     <row r="53" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="29" t="s">
-        <v>27</v>
-      </c>
-      <c r="B53" s="27" t="s">
-        <v>28</v>
+        <v>26</v>
+      </c>
+      <c r="B53" s="30" t="s">
+        <v>78</v>
       </c>
       <c r="C53" s="2" t="s">
         <v>13</v>
@@ -2193,17 +2222,23 @@
       <c r="D53" s="3">
         <v>9.5</v>
       </c>
-      <c r="E53" s="4"/>
-      <c r="F53" s="5" t="str">
+      <c r="E53" s="4">
+        <v>9.9600000000000009</v>
+      </c>
+      <c r="F53" s="5">
         <f>IF(E53="","",E53-D53)</f>
-        <v/>
+        <v>0.46000000000000085</v>
       </c>
       <c r="G53" s="6" t="str">
         <f>IF(E53="","",IF(AND(E53&gt;=9,E53&lt;=10),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H53" s="7"/>
-      <c r="I53" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H53" s="7">
+        <v>1</v>
+      </c>
+      <c r="I53" s="8">
+        <v>0.99</v>
+      </c>
     </row>
     <row r="54" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="28"/>
@@ -2214,17 +2249,23 @@
       <c r="D54" s="3">
         <v>7.5</v>
       </c>
-      <c r="E54" s="4"/>
-      <c r="F54" s="5" t="str">
+      <c r="E54" s="4">
+        <v>9.59</v>
+      </c>
+      <c r="F54" s="5">
         <f>IF(E54="","",E54-D54)</f>
-        <v/>
+        <v>2.09</v>
       </c>
       <c r="G54" s="6" t="str">
         <f>IF(E54="","",IF(AND(E54&gt;=7,E54&lt;=9),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H54" s="7"/>
-      <c r="I54" s="8"/>
+        <v>✗ No</v>
+      </c>
+      <c r="H54" s="7">
+        <v>0.93</v>
+      </c>
+      <c r="I54" s="8">
+        <v>0.99</v>
+      </c>
     </row>
     <row r="55" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="28"/>
@@ -2235,17 +2276,23 @@
       <c r="D55" s="3">
         <v>5.5</v>
       </c>
-      <c r="E55" s="4"/>
-      <c r="F55" s="5" t="str">
+      <c r="E55" s="4">
+        <v>6.51</v>
+      </c>
+      <c r="F55" s="5">
         <f>IF(E55="","",E55-D55)</f>
-        <v/>
+        <v>1.0099999999999998</v>
       </c>
       <c r="G55" s="6" t="str">
         <f>IF(E55="","",IF(AND(E55&gt;=4.5,E55&lt;=7),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H55" s="7"/>
-      <c r="I55" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H55" s="7">
+        <v>0.78</v>
+      </c>
+      <c r="I55" s="8">
+        <v>0.92</v>
+      </c>
     </row>
     <row r="56" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="28"/>
@@ -2256,17 +2303,23 @@
       <c r="D56" s="3">
         <v>3.5</v>
       </c>
-      <c r="E56" s="4"/>
-      <c r="F56" s="5" t="str">
+      <c r="E56" s="4">
+        <v>4.17</v>
+      </c>
+      <c r="F56" s="5">
         <f>IF(E56="","",E56-D56)</f>
-        <v/>
+        <v>0.66999999999999993</v>
       </c>
       <c r="G56" s="6" t="str">
         <f>IF(E56="","",IF(AND(E56&gt;=2.5,E56&lt;=4.5),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H56" s="7"/>
-      <c r="I56" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H56" s="7">
+        <v>0.72</v>
+      </c>
+      <c r="I56" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="57" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="28"/>
@@ -2277,17 +2330,23 @@
       <c r="D57" s="3">
         <v>1.5</v>
       </c>
-      <c r="E57" s="4"/>
-      <c r="F57" s="5" t="str">
+      <c r="E57" s="4">
+        <v>4.1100000000000003</v>
+      </c>
+      <c r="F57" s="5">
         <f>IF(E57="","",E57-D57)</f>
-        <v/>
+        <v>2.6100000000000003</v>
       </c>
       <c r="G57" s="6" t="str">
         <f>IF(E57="","",IF(AND(E57&gt;=0,E57&lt;=2.5),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H57" s="7"/>
-      <c r="I57" s="8"/>
+        <v>✗ No</v>
+      </c>
+      <c r="H57" s="7">
+        <v>0.7</v>
+      </c>
+      <c r="I57" s="8">
+        <v>0</v>
+      </c>
     </row>
     <row r="58" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="13"/>
@@ -2302,10 +2361,10 @@
     </row>
     <row r="59" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="29" t="s">
-        <v>29</v>
-      </c>
-      <c r="B59" s="27" t="s">
-        <v>30</v>
+        <v>27</v>
+      </c>
+      <c r="B59" s="30" t="s">
+        <v>79</v>
       </c>
       <c r="C59" s="2" t="s">
         <v>13</v>
@@ -2313,17 +2372,23 @@
       <c r="D59" s="3">
         <v>9.5</v>
       </c>
-      <c r="E59" s="4"/>
-      <c r="F59" s="5" t="str">
+      <c r="E59" s="4">
+        <v>9.7899999999999991</v>
+      </c>
+      <c r="F59" s="5">
         <f>IF(E59="","",E59-D59)</f>
-        <v/>
+        <v>0.28999999999999915</v>
       </c>
       <c r="G59" s="6" t="str">
         <f>IF(E59="","",IF(AND(E59&gt;=9,E59&lt;=10),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H59" s="7"/>
-      <c r="I59" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H59" s="7">
+        <v>0.96</v>
+      </c>
+      <c r="I59" s="8">
+        <v>0.99</v>
+      </c>
     </row>
     <row r="60" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="28"/>
@@ -2334,17 +2399,23 @@
       <c r="D60" s="3">
         <v>7.5</v>
       </c>
-      <c r="E60" s="4"/>
-      <c r="F60" s="5" t="str">
+      <c r="E60" s="4">
+        <v>6.44</v>
+      </c>
+      <c r="F60" s="5">
         <f>IF(E60="","",E60-D60)</f>
-        <v/>
+        <v>-1.0599999999999996</v>
       </c>
       <c r="G60" s="6" t="str">
         <f>IF(E60="","",IF(AND(E60&gt;=7,E60&lt;=9),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H60" s="7"/>
-      <c r="I60" s="8"/>
+        <v>✗ No</v>
+      </c>
+      <c r="H60" s="7">
+        <v>0.74</v>
+      </c>
+      <c r="I60" s="8">
+        <v>0.97</v>
+      </c>
     </row>
     <row r="61" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A61" s="28"/>
@@ -2355,17 +2426,23 @@
       <c r="D61" s="3">
         <v>5.5</v>
       </c>
-      <c r="E61" s="4"/>
-      <c r="F61" s="5" t="str">
+      <c r="E61" s="4">
+        <v>5.26</v>
+      </c>
+      <c r="F61" s="5">
         <f>IF(E61="","",E61-D61)</f>
-        <v/>
+        <v>-0.24000000000000021</v>
       </c>
       <c r="G61" s="6" t="str">
         <f>IF(E61="","",IF(AND(E61&gt;=4.5,E61&lt;=7),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H61" s="7"/>
-      <c r="I61" s="8"/>
+        <v>✓ Yes</v>
+      </c>
+      <c r="H61" s="7">
+        <v>0.86</v>
+      </c>
+      <c r="I61" s="8">
+        <v>0.17</v>
+      </c>
     </row>
     <row r="62" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A62" s="28"/>
@@ -2376,17 +2453,23 @@
       <c r="D62" s="3">
         <v>3.5</v>
       </c>
-      <c r="E62" s="4"/>
-      <c r="F62" s="5" t="str">
+      <c r="E62" s="4">
+        <v>4.63</v>
+      </c>
+      <c r="F62" s="5">
         <f>IF(E62="","",E62-D62)</f>
-        <v/>
+        <v>1.1299999999999999</v>
       </c>
       <c r="G62" s="6" t="str">
         <f>IF(E62="","",IF(AND(E62&gt;=2.5,E62&lt;=4.5),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H62" s="7"/>
-      <c r="I62" s="8"/>
+        <v>✗ No</v>
+      </c>
+      <c r="H62" s="7">
+        <v>0.8</v>
+      </c>
+      <c r="I62" s="8">
+        <v>0.19</v>
+      </c>
     </row>
     <row r="63" spans="1:9" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A63" s="28"/>
@@ -2397,17 +2480,23 @@
       <c r="D63" s="3">
         <v>1.5</v>
       </c>
-      <c r="E63" s="4"/>
-      <c r="F63" s="5" t="str">
+      <c r="E63" s="4">
+        <v>3.67</v>
+      </c>
+      <c r="F63" s="5">
         <f>IF(E63="","",E63-D63)</f>
-        <v/>
+        <v>2.17</v>
       </c>
       <c r="G63" s="6" t="str">
         <f>IF(E63="","",IF(AND(E63&gt;=0,E63&lt;=2.5),"✓ Yes","✗ No"))</f>
-        <v/>
-      </c>
-      <c r="H63" s="7"/>
-      <c r="I63" s="8"/>
+        <v>✗ No</v>
+      </c>
+      <c r="H63" s="7">
+        <v>0.77</v>
+      </c>
+      <c r="I63" s="8">
+        <v>0.01</v>
+      </c>
     </row>
     <row r="64" spans="1:9" ht="6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A64" s="13"/>
@@ -2422,6 +2511,13 @@
     </row>
   </sheetData>
   <mergeCells count="22">
+    <mergeCell ref="A59:A63"/>
+    <mergeCell ref="B41:B45"/>
+    <mergeCell ref="B59:B63"/>
+    <mergeCell ref="B35:B39"/>
+    <mergeCell ref="B47:B51"/>
+    <mergeCell ref="B53:B57"/>
+    <mergeCell ref="A47:A51"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A41:A45"/>
     <mergeCell ref="B23:B27"/>
@@ -2429,18 +2525,11 @@
     <mergeCell ref="A53:A57"/>
     <mergeCell ref="A29:A33"/>
     <mergeCell ref="A35:A39"/>
-    <mergeCell ref="A59:A63"/>
-    <mergeCell ref="B41:B45"/>
-    <mergeCell ref="B59:B63"/>
-    <mergeCell ref="B35:B39"/>
-    <mergeCell ref="B47:B51"/>
     <mergeCell ref="A11:A15"/>
     <mergeCell ref="B17:B21"/>
     <mergeCell ref="B11:B15"/>
-    <mergeCell ref="B53:B57"/>
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="B29:B33"/>
-    <mergeCell ref="A47:A51"/>
     <mergeCell ref="A23:A27"/>
     <mergeCell ref="B5:B9"/>
     <mergeCell ref="A17:A21"/>
@@ -2462,8 +2551,8 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>31</v>
+      <c r="A1" s="36" t="s">
+        <v>28</v>
       </c>
       <c r="B1" s="28"/>
       <c r="C1" s="28"/>
@@ -2473,8 +2562,8 @@
       <c r="G1" s="28"/>
     </row>
     <row r="2" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="36" t="s">
-        <v>32</v>
+      <c r="A2" s="34" t="s">
+        <v>29</v>
       </c>
       <c r="B2" s="28"/>
       <c r="C2" s="28"/>
@@ -2485,8 +2574,8 @@
     </row>
     <row r="3" spans="1:7" ht="10.050000000000001" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="4" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="32" t="s">
-        <v>33</v>
+      <c r="A4" s="33" t="s">
+        <v>30</v>
       </c>
       <c r="B4" s="28"/>
       <c r="C4" s="28"/>
@@ -2500,22 +2589,22 @@
         <v>4</v>
       </c>
       <c r="B5" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="14" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="14" t="s">
         <v>34</v>
       </c>
-      <c r="C5" s="14" t="s">
+      <c r="F5" s="14" t="s">
         <v>35</v>
       </c>
-      <c r="D5" s="14" t="s">
+      <c r="G5" s="14" t="s">
         <v>36</v>
-      </c>
-      <c r="E5" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="F5" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="G5" s="14" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2527,11 +2616,11 @@
       </c>
       <c r="C6" s="16">
         <f>IFERROR(AVERAGE('Score Entry'!E5,'Score Entry'!E11,'Score Entry'!E17,'Score Entry'!E23,'Score Entry'!E29,'Score Entry'!E35,'Score Entry'!E41,'Score Entry'!E47,'Score Entry'!E53,'Score Entry'!E59),"Fill scores")</f>
-        <v>8.6085714285714285</v>
+        <v>8.9779999999999998</v>
       </c>
       <c r="D6" s="17">
         <f>IFERROR(STDEV('Score Entry'!E5,'Score Entry'!E11,'Score Entry'!E17,'Score Entry'!E23,'Score Entry'!E29,'Score Entry'!E35,'Score Entry'!E41,'Score Entry'!E47,'Score Entry'!E53,'Score Entry'!E59),"")</f>
-        <v>0.89411834733866136</v>
+        <v>0.94298344512392029</v>
       </c>
       <c r="E6" s="17">
         <f>IFERROR(MIN('Score Entry'!E5,'Score Entry'!E11,'Score Entry'!E17,'Score Entry'!E23,'Score Entry'!E29,'Score Entry'!E35,'Score Entry'!E41,'Score Entry'!E47,'Score Entry'!E53,'Score Entry'!E59),"")</f>
@@ -2539,7 +2628,7 @@
       </c>
       <c r="F6" s="17">
         <f>IFERROR(MAX('Score Entry'!E5,'Score Entry'!E11,'Score Entry'!E17,'Score Entry'!E23,'Score Entry'!E29,'Score Entry'!E35,'Score Entry'!E41,'Score Entry'!E47,'Score Entry'!E53,'Score Entry'!E59),"")</f>
-        <v>9.93</v>
+        <v>9.9600000000000009</v>
       </c>
       <c r="G6" s="18"/>
     </row>
@@ -2552,11 +2641,11 @@
       </c>
       <c r="C7" s="16">
         <f>IFERROR(AVERAGE('Score Entry'!E6,'Score Entry'!E12,'Score Entry'!E18,'Score Entry'!E24,'Score Entry'!E30,'Score Entry'!E36,'Score Entry'!E42,'Score Entry'!E48,'Score Entry'!E54,'Score Entry'!E60),"Fill scores")</f>
-        <v>6.9157142857142855</v>
+        <v>7.1579999999999995</v>
       </c>
       <c r="D7" s="17">
         <f>IFERROR(STDEV('Score Entry'!E6,'Score Entry'!E12,'Score Entry'!E18,'Score Entry'!E24,'Score Entry'!E30,'Score Entry'!E36,'Score Entry'!E42,'Score Entry'!E48,'Score Entry'!E54,'Score Entry'!E60),"")</f>
-        <v>0.76508947500400615</v>
+        <v>1.0725649423487347</v>
       </c>
       <c r="E7" s="17">
         <f>IFERROR(MIN('Score Entry'!E6,'Score Entry'!E12,'Score Entry'!E18,'Score Entry'!E24,'Score Entry'!E30,'Score Entry'!E36,'Score Entry'!E42,'Score Entry'!E48,'Score Entry'!E54,'Score Entry'!E60),"")</f>
@@ -2564,7 +2653,7 @@
       </c>
       <c r="F7" s="17">
         <f>IFERROR(MAX('Score Entry'!E6,'Score Entry'!E12,'Score Entry'!E18,'Score Entry'!E24,'Score Entry'!E30,'Score Entry'!E36,'Score Entry'!E42,'Score Entry'!E48,'Score Entry'!E54,'Score Entry'!E60),"")</f>
-        <v>7.9</v>
+        <v>9.59</v>
       </c>
       <c r="G7" s="18"/>
     </row>
@@ -2577,11 +2666,11 @@
       </c>
       <c r="C8" s="16">
         <f>IFERROR(AVERAGE('Score Entry'!E7,'Score Entry'!E13,'Score Entry'!E19,'Score Entry'!E25,'Score Entry'!E31,'Score Entry'!E37,'Score Entry'!E43,'Score Entry'!E49,'Score Entry'!E55,'Score Entry'!E61),"Fill scores")</f>
-        <v>5.7728571428571422</v>
+        <v>5.9359999999999991</v>
       </c>
       <c r="D8" s="17">
         <f>IFERROR(STDEV('Score Entry'!E7,'Score Entry'!E13,'Score Entry'!E19,'Score Entry'!E25,'Score Entry'!E31,'Score Entry'!E37,'Score Entry'!E43,'Score Entry'!E49,'Score Entry'!E55,'Score Entry'!E61),"")</f>
-        <v>0.84332109910192632</v>
+        <v>0.86842385964459734</v>
       </c>
       <c r="E8" s="17">
         <f>IFERROR(MIN('Score Entry'!E7,'Score Entry'!E13,'Score Entry'!E19,'Score Entry'!E25,'Score Entry'!E31,'Score Entry'!E37,'Score Entry'!E43,'Score Entry'!E49,'Score Entry'!E55,'Score Entry'!E61),"")</f>
@@ -2589,7 +2678,7 @@
       </c>
       <c r="F8" s="17">
         <f>IFERROR(MAX('Score Entry'!E7,'Score Entry'!E13,'Score Entry'!E19,'Score Entry'!E25,'Score Entry'!E31,'Score Entry'!E37,'Score Entry'!E43,'Score Entry'!E49,'Score Entry'!E55,'Score Entry'!E61),"")</f>
-        <v>7.02</v>
+        <v>7.18</v>
       </c>
       <c r="G8" s="18"/>
     </row>
@@ -2602,11 +2691,11 @@
       </c>
       <c r="C9" s="16">
         <f>IFERROR(AVERAGE('Score Entry'!E8,'Score Entry'!E14,'Score Entry'!E20,'Score Entry'!E26,'Score Entry'!E32,'Score Entry'!E38,'Score Entry'!E44,'Score Entry'!E50,'Score Entry'!E56,'Score Entry'!E62),"Fill scores")</f>
-        <v>4.1757142857142853</v>
+        <v>4.4779999999999998</v>
       </c>
       <c r="D9" s="17">
         <f>IFERROR(STDEV('Score Entry'!E8,'Score Entry'!E14,'Score Entry'!E20,'Score Entry'!E26,'Score Entry'!E32,'Score Entry'!E38,'Score Entry'!E44,'Score Entry'!E50,'Score Entry'!E56,'Score Entry'!E62),"")</f>
-        <v>1.3744921139928659</v>
+        <v>1.3846363341245163</v>
       </c>
       <c r="E9" s="17">
         <f>IFERROR(MIN('Score Entry'!E8,'Score Entry'!E14,'Score Entry'!E20,'Score Entry'!E26,'Score Entry'!E32,'Score Entry'!E38,'Score Entry'!E44,'Score Entry'!E50,'Score Entry'!E56,'Score Entry'!E62),"")</f>
@@ -2614,7 +2703,7 @@
       </c>
       <c r="F9" s="17">
         <f>IFERROR(MAX('Score Entry'!E8,'Score Entry'!E14,'Score Entry'!E20,'Score Entry'!E26,'Score Entry'!E32,'Score Entry'!E38,'Score Entry'!E44,'Score Entry'!E50,'Score Entry'!E56,'Score Entry'!E62),"")</f>
-        <v>6.18</v>
+        <v>6.75</v>
       </c>
       <c r="G9" s="18"/>
     </row>
@@ -2627,15 +2716,15 @@
       </c>
       <c r="C10" s="16">
         <f>IFERROR(AVERAGE('Score Entry'!E9,'Score Entry'!E15,'Score Entry'!E21,'Score Entry'!E27,'Score Entry'!E33,'Score Entry'!E39,'Score Entry'!E45,'Score Entry'!E51,'Score Entry'!E57,'Score Entry'!E63),"Fill scores")</f>
-        <v>3.5457142857142858</v>
+        <v>3.2619999999999996</v>
       </c>
       <c r="D10" s="17">
         <f>IFERROR(STDEV('Score Entry'!E9,'Score Entry'!E15,'Score Entry'!E21,'Score Entry'!E27,'Score Entry'!E33,'Score Entry'!E39,'Score Entry'!E45,'Score Entry'!E51,'Score Entry'!E57,'Score Entry'!E63),"")</f>
-        <v>0.46050179669780117</v>
+        <v>1.2125253720140379</v>
       </c>
       <c r="E10" s="17">
         <f>IFERROR(MIN('Score Entry'!E9,'Score Entry'!E15,'Score Entry'!E21,'Score Entry'!E27,'Score Entry'!E33,'Score Entry'!E39,'Score Entry'!E45,'Score Entry'!E51,'Score Entry'!E57,'Score Entry'!E63),"")</f>
-        <v>3.11</v>
+        <v>0.02</v>
       </c>
       <c r="F10" s="17">
         <f>IFERROR(MAX('Score Entry'!E9,'Score Entry'!E15,'Score Entry'!E21,'Score Entry'!E27,'Score Entry'!E33,'Score Entry'!E39,'Score Entry'!E45,'Score Entry'!E51,'Score Entry'!E57,'Score Entry'!E63),"")</f>
@@ -2645,8 +2734,8 @@
     </row>
     <row r="12" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="1:7" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="32" t="s">
-        <v>40</v>
+      <c r="A13" s="33" t="s">
+        <v>37</v>
       </c>
       <c r="B13" s="28"/>
       <c r="C13" s="28"/>
@@ -2656,8 +2745,8 @@
       <c r="G13" s="28"/>
     </row>
     <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="33" t="s">
-        <v>41</v>
+      <c r="A14" s="35" t="s">
+        <v>38</v>
       </c>
       <c r="B14" s="28"/>
       <c r="C14" s="28"/>
@@ -2668,10 +2757,10 @@
     </row>
     <row r="15" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="23" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="34" t="s">
-        <v>43</v>
+        <v>39</v>
+      </c>
+      <c r="B15" s="32" t="s">
+        <v>40</v>
       </c>
       <c r="C15" s="28"/>
       <c r="D15" s="28"/>
@@ -2681,10 +2770,10 @@
     </row>
     <row r="16" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="23" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="34" t="s">
-        <v>45</v>
+        <v>41</v>
+      </c>
+      <c r="B16" s="32" t="s">
+        <v>42</v>
       </c>
       <c r="C16" s="28"/>
       <c r="D16" s="28"/>
@@ -2694,10 +2783,10 @@
     </row>
     <row r="17" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="23" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="34" t="s">
-        <v>47</v>
+        <v>43</v>
+      </c>
+      <c r="B17" s="32" t="s">
+        <v>44</v>
       </c>
       <c r="C17" s="28"/>
       <c r="D17" s="28"/>
@@ -2707,10 +2796,10 @@
     </row>
     <row r="18" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="23" t="s">
-        <v>48</v>
-      </c>
-      <c r="B18" s="34" t="s">
-        <v>49</v>
+        <v>45</v>
+      </c>
+      <c r="B18" s="32" t="s">
+        <v>46</v>
       </c>
       <c r="C18" s="28"/>
       <c r="D18" s="28"/>
@@ -2720,10 +2809,10 @@
     </row>
     <row r="19" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="23" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" s="34" t="s">
-        <v>51</v>
+        <v>47</v>
+      </c>
+      <c r="B19" s="32" t="s">
+        <v>48</v>
       </c>
       <c r="C19" s="28"/>
       <c r="D19" s="28"/>
@@ -2733,10 +2822,10 @@
     </row>
     <row r="20" spans="1:7" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="23" t="s">
-        <v>52</v>
-      </c>
-      <c r="B20" s="34" t="s">
-        <v>53</v>
+        <v>49</v>
+      </c>
+      <c r="B20" s="32" t="s">
+        <v>50</v>
       </c>
       <c r="C20" s="28"/>
       <c r="D20" s="28"/>
@@ -2746,6 +2835,7 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A1:G1"/>
     <mergeCell ref="B20:G20"/>
     <mergeCell ref="B17:G17"/>
     <mergeCell ref="A4:G4"/>
@@ -2756,7 +2846,6 @@
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="B16:G16"/>
     <mergeCell ref="B19:G19"/>
-    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2772,65 +2861,65 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="35" t="s">
-        <v>54</v>
+      <c r="A1" s="36" t="s">
+        <v>51</v>
       </c>
       <c r="B1" s="28"/>
     </row>
     <row r="3" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="25" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B3" s="24" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="25" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="B4" s="24" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="25" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B5" s="24" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="25" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B6" s="24" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="25" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B7" s="24" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="25" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B8" s="24" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="25" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B9" s="24" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -2839,7 +2928,7 @@
     </row>
     <row r="11" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="26" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B11" s="24" t="e">
         <f>AI Score input — MUST fill these (Column E in Score Entry)</f>
@@ -2848,13 +2937,13 @@
     </row>
     <row r="12" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="26" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B12" s="24"/>
     </row>
     <row r="13" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="26" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B13" s="24"/>
     </row>
@@ -2864,18 +2953,18 @@
     </row>
     <row r="15" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B15" s="24" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
     </row>
     <row r="16" spans="1:2" ht="22.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="26" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="B16" s="24" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>